<commit_message>
Fixed hitlocations and weapons for Walktapus
</commit_message>
<xml_diff>
--- a/Data/weapons_melee_table.xlsx
+++ b/Data/weapons_melee_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\Stat_blocks\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7563EC1D-6DEC-46CF-AC8B-1A2C1BA8D0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDE12E8-BCCA-4B87-B1B2-0B45EA46B4D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="2340" windowWidth="32175" windowHeight="19260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="1620" windowWidth="32175" windowHeight="19260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="119">
   <si>
     <t>Name</t>
   </si>
@@ -349,9 +349,6 @@
     <t>Auto Poison,</t>
   </si>
   <si>
-    <t>POT=CON</t>
-  </si>
-  <si>
     <t>1D4-1</t>
   </si>
   <si>
@@ -377,6 +374,9 @@
   </si>
   <si>
     <t>Giant Honeybee Queen</t>
+  </si>
+  <si>
+    <t>Auto</t>
   </si>
 </sst>
 </file>
@@ -723,7 +723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.83203125" customWidth="1"/>
@@ -1721,7 +1721,7 @@
         <v>101</v>
       </c>
       <c r="B54">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="C54" t="s">
         <v>89</v>
@@ -1740,8 +1740,8 @@
       <c r="A55" t="s">
         <v>104</v>
       </c>
-      <c r="B55">
-        <v>0</v>
+      <c r="B55" t="s">
+        <v>118</v>
       </c>
       <c r="C55" t="s">
         <v>89</v>
@@ -1760,8 +1760,8 @@
       <c r="A56" t="s">
         <v>106</v>
       </c>
-      <c r="B56">
-        <v>0</v>
+      <c r="B56" t="s">
+        <v>118</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -1781,19 +1781,28 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
+        <v>70</v>
+      </c>
+      <c r="B57">
+        <v>20</v>
+      </c>
+      <c r="C57" t="s">
         <v>109</v>
       </c>
-      <c r="B57">
-        <v>1</v>
-      </c>
       <c r="E57">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F57" t="s">
-        <v>102</v>
+        <v>110</v>
+      </c>
+      <c r="G57" t="s">
+        <v>70</v>
+      </c>
+      <c r="H57" t="s">
+        <v>111</v>
       </c>
       <c r="J57" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
@@ -1801,30 +1810,30 @@
         <v>70</v>
       </c>
       <c r="B58">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C58" t="s">
-        <v>110</v>
+        <v>11</v>
       </c>
       <c r="E58">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F58" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G58" t="s">
         <v>70</v>
       </c>
       <c r="H58" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J58" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B59">
         <v>30</v>
@@ -1836,21 +1845,21 @@
         <v>0</v>
       </c>
       <c r="F59" t="s">
+        <v>113</v>
+      </c>
+      <c r="G59" t="s">
+        <v>71</v>
+      </c>
+      <c r="H59" t="s">
         <v>114</v>
       </c>
-      <c r="G59" t="s">
-        <v>70</v>
-      </c>
-      <c r="H59" t="s">
+      <c r="J59" t="s">
         <v>115</v>
-      </c>
-      <c r="J59" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B60">
         <v>30</v>
@@ -1862,16 +1871,16 @@
         <v>0</v>
       </c>
       <c r="F60" t="s">
+        <v>116</v>
+      </c>
+      <c r="G60" t="s">
+        <v>70</v>
+      </c>
+      <c r="H60" t="s">
         <v>114</v>
       </c>
-      <c r="G60" t="s">
-        <v>71</v>
-      </c>
-      <c r="H60" t="s">
+      <c r="J60" t="s">
         <v>115</v>
-      </c>
-      <c r="J60" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
@@ -1879,7 +1888,7 @@
         <v>70</v>
       </c>
       <c r="B61">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="C61" t="s">
         <v>11</v>
@@ -1894,15 +1903,15 @@
         <v>70</v>
       </c>
       <c r="H61" t="s">
+        <v>114</v>
+      </c>
+      <c r="J61" t="s">
         <v>115</v>
-      </c>
-      <c r="J61" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B62">
         <v>80</v>
@@ -1914,42 +1923,16 @@
         <v>0</v>
       </c>
       <c r="F62" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G62" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H62" t="s">
+        <v>114</v>
+      </c>
+      <c r="J62" t="s">
         <v>115</v>
-      </c>
-      <c r="J62" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>71</v>
-      </c>
-      <c r="B63">
-        <v>80</v>
-      </c>
-      <c r="C63" t="s">
-        <v>11</v>
-      </c>
-      <c r="E63">
-        <v>0</v>
-      </c>
-      <c r="F63" t="s">
-        <v>118</v>
-      </c>
-      <c r="G63" t="s">
-        <v>71</v>
-      </c>
-      <c r="H63" t="s">
-        <v>115</v>
-      </c>
-      <c r="J63" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>